<commit_message>
correction consumable.manufacturedProduct et typeCode code-barres c04442a0954e04d54bbc911d9cefd7a306f73c7b
</commit_message>
<xml_diff>
--- a/fix/slicing-type-this/ig/StructureDefinition-fr-cda-code-a-barres.xlsx
+++ b/fix/slicing-type-this/ig/StructureDefinition-fr-cda-code-a-barres.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-07T08:37:44+00:00</t>
+    <t>2026-10-07T09:51:04+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -6410,7 +6410,7 @@
       </c>
       <c r="E51" s="2"/>
       <c r="F51" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G51" t="s" s="2">
         <v>76</v>

</xml_diff>